<commit_message>
Time stamp fixed instant refresh fixed
</commit_message>
<xml_diff>
--- a/ExportedReports/Tasks_All_Users_All_Time.xlsx
+++ b/ExportedReports/Tasks_All_Users_All_Time.xlsx
@@ -19,7 +19,7 @@
     <x:t>Task Management System — Export Report</x:t>
   </x:si>
   <x:si>
-    <x:t>Filters: User: All Users | Period: All | Exported: 2026-10-21 02:32 UTC | Total: 31</x:t>
+    <x:t>Filters: User: All Users | Period: All | Exported: 2026-10-21 05:50 AM (Egypt Time) | Total: 31</x:t>
   </x:si>
   <x:si>
     <x:t>Task #</x:t>
@@ -46,13 +46,13 @@
     <x:t>johndoe_test@example.com</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-21 02:16</x:t>
+    <x:t>2026-10-21 05:16 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Design Flutter Dashboard] Created mockup and flutter widget tree for dashboard.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-21 02:15</x:t>
+    <x:t>2026-10-21 05:15 AM</x:t>
   </x:si>
   <x:si>
     <x:t>Alex Mercer</x:t>
@@ -61,10 +61,10 @@
     <x:t>alex.mercer@tasksystem.com</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-21 01:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-21 01:52</x:t>
+    <x:t>2026-10-21 04:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-21 04:52 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[End-to-End API Integration Suite] Wrote automated PowerShell integration test script covering registration, JWT issuance, multi-date task logging, timeframe assertions, and Excel file validation.</x:t>
@@ -76,10 +76,10 @@
     <x:t>sarah.connor@tasksystem.com</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-20 23:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-21 00:32</x:t>
+    <x:t>2026-10-21 02:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-21 03:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Flutter Task Submission UI] Designed and developed the Flutter form screen allowing employees to enter task descriptions, select completed timestamps, and submit to the backend API.</x:t>
@@ -91,10 +91,10 @@
     <x:t>elena.rostova@tasksystem.com</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-20 20:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-20 21:32</x:t>
+    <x:t>2026-10-20 11:32 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-21 12:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Excel Export with ClosedXML] Architected high-performance Excel report builder utilizing ClosedXML. Added alternating row fills, thin gray borders, title banner, and streaming download response.</x:t>
@@ -106,10 +106,10 @@
     <x:t>tariq.mansour@tasksystem.com</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-20 16:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-20 17:32</x:t>
+    <x:t>2026-10-20 07:32 PM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-20 08:32 PM</x:t>
   </x:si>
   <x:si>
     <x:t>[Admin Dashboard UX Redesign] Created polished Bootstrap 5 layout featuring clean filter cards, status badges, responsive navigation bar, and high-contrast readable typography.</x:t>
@@ -121,196 +121,196 @@
     <x:t>michael.scott@tasksystem.com</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-20 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-20 03:32</x:t>
+    <x:t>2026-10-20 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-20 06:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Sprint 14 Planning &amp; Review] Conducted bi-weekly sprint planning meeting with engineering team. Groomed backlog user stories, assigned story points, and resolved feature dependencies.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-19 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-19 04:32</x:t>
+    <x:t>2026-10-19 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-19 07:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Load Testing on Excel Export] Simulated simultaneous export requests for large task datasets (10,000+ records) to verify memory stability and response latency under 500ms.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-19 03:32</x:t>
+    <x:t>2026-10-19 06:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Secure JWT Storage in Flutter] Integrated flutter_secure_storage package to store authentication tokens and automatically attach Authorization Bearer headers to HTTP interceptors.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-18 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-18 03:32</x:t>
+    <x:t>2026-10-18 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-18 06:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Dynamic Query Filtering Engine] Implemented reusable repository expressions to dynamically filter task submissions by timeframe preset (week/month/year) and explicit start/end dates.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-17 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-17 05:32</x:t>
+    <x:t>2026-10-17 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-17 08:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Mobile Dark Mode Theme] Built Figma design system for Flutter mobile dark and light themes, including custom color palettes for status badges and cards.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-17 02:16</x:t>
+    <x:t>2026-10-17 05:16 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Implement Authentication Service] Wrote Flutter secure storage and JWT handling logic.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-17 02:15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-16 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-16 04:32</x:t>
+    <x:t>2026-10-17 05:15 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-16 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-16 07:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[State Management with Bloc] Refactored user task history view to use flutter_bloc. Handled loading, loaded, and network failure states with custom retry widgets.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-15 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-15 04:32</x:t>
+    <x:t>2026-10-15 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-15 07:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Client Demonstration &amp; Walkthrough] Presented interactive live demo of the Task Management Mobile App and Admin Dashboard to executive stakeholders. Gathered positive feedback on reporting speed.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-10 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-10 06:32</x:t>
+    <x:t>2026-10-10 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-10 09:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Mobile Cross-Platform Smoke Testing] Executed automated smoke test suite across 4 Android emulator devices and 2 iOS simulators to verify responsive UI rendering.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-09 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-09 03:02</x:t>
+    <x:t>2026-10-09 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-09 06:02 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[SQL Index Optimization] Analyzed execution plans on Tasks table. Added B-Tree composite indices on (UserId) and (TaskDate) to ensure millisecond queries over millions of records.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-06 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-06 04:32</x:t>
+    <x:t>2026-10-06 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-06 07:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Iconography &amp; Accessibility Polish] Audited color contrast ratios according to WCAG 2.1 AA guidelines. Updated button focus states and screen reader aria labels across admin views.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-03 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-10-03 03:17</x:t>
+    <x:t>2026-10-03 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-03 06:17 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Offline Task Sync Service] Added SQLite local database caching so employees can log tasks even while offline and batch-sync them once network connection restores.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-01 02:16</x:t>
+    <x:t>2026-10-01 05:16 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Database &amp; Repository Layer] Designed relational schema and configured Entity Framework Core.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-01 02:15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-09-29 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-09-29 05:32</x:t>
+    <x:t>2026-10-01 05:15 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-09-29 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-09-29 08:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Q4 Milestone Audit] Audited project deliverables against Q4 target roadmap. Verified all planned authentication, mobile submission, and spreadsheet features are on track.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-09-26 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-09-26 04:32</x:t>
+    <x:t>2026-09-26 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-09-26 07:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Dual Authentication Pipeline] Configured ASP.NET Core middleware to simultaneously support JWT Bearer tokens for mobile clients and Cookie sessions for web admin dashboard.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-09-01 02:16</x:t>
+    <x:t>2026-09-01 05:16 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Architecture Setup] Initial requirement gathering and solution architecture definition.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-09-01 02:15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-08-07 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-08-07 05:32</x:t>
+    <x:t>2026-09-01 05:15 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-08-07 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-08-07 08:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Android &amp; iOS App Signing] Configured keystores, provisioning profiles, and automated Fastlane pipelines for staging deployment builds.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-07-23 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-07-23 07:32</x:t>
+    <x:t>2026-07-23 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-23 10:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Design System Component Library] Created reusable Figma UI kit with 40+ components, form inputs, date pickers, dropdowns, and data table layouts.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-06-03 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-03 06:32</x:t>
+    <x:t>2026-06-03 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-03 09:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Database Migration &amp; Seed Script] Constructed Entity Framework Core Code-First migrations and automated DB initializer with role management and admin provisioning.</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-03-25 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-03-25 03:32</x:t>
+    <x:t>2026-03-25 04:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-03-25 05:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Security &amp; Compliance Review] Reviewed GDPR compliance requirements, password hashing standards, and data retention policies for submitted employee logs.</x:t>
   </x:si>
   <x:si>
-    <x:t>2025-12-05 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2025-12-05 03:32</x:t>
+    <x:t>2025-12-05 04:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2025-12-05 05:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Regression Test Suite v1.0] Documented complete test matrix covering token refresh scenarios, expired credentials, invalid date ranges, and SQL injection protections.</x:t>
   </x:si>
   <x:si>
-    <x:t>2025-07-28 02:32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2025-07-28 04:32</x:t>
+    <x:t>2025-07-28 05:32 AM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2025-07-28 07:32 AM</x:t>
   </x:si>
   <x:si>
     <x:t>[Historical Archive Legacy Test] Archived legacy task records from previous fiscal year to ensure backwards compatibility with historical data imports.</x:t>
@@ -844,7 +844,8 @@
   <x:cols>
     <x:col min="1" max="1" width="10.710625" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="24.710625" style="0" customWidth="1"/>
-    <x:col min="3" max="5" width="28.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28.710625" style="0" customWidth="1"/>
+    <x:col min="4" max="5" width="30.710625" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="50.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>

</xml_diff>